<commit_message>
Age Groups: Team settings
</commit_message>
<xml_diff>
--- a/local/agegroups/2026-Nationals.xlsx
+++ b/local/agegroups/2026-Nationals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/agegroups/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898DC0C6-0DF4-D74B-9B4F-115E16172D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288BED6D-637A-E446-BEDD-9AB414738E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21880" yWindow="5240" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -4342,10 +4342,16 @@
         <v>58</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N2">
         <v>2</v>
+      </c>
+      <c r="O2">
+        <v>5</v>
+      </c>
+      <c r="P2">
+        <v>5</v>
       </c>
       <c r="Q2" s="1"/>
       <c r="R2" t="b">
@@ -4387,10 +4393,16 @@
         <v>58</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N3">
         <v>2</v>
+      </c>
+      <c r="O3">
+        <v>5</v>
+      </c>
+      <c r="P3">
+        <v>5</v>
       </c>
       <c r="Q3" s="1"/>
       <c r="R3" t="b">
@@ -4432,10 +4444,16 @@
         <v>58</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N4">
         <v>2</v>
+      </c>
+      <c r="O4">
+        <v>5</v>
+      </c>
+      <c r="P4">
+        <v>5</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="R4" t="b">
@@ -4477,10 +4495,16 @@
         <v>58</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N5">
         <v>2</v>
+      </c>
+      <c r="O5">
+        <v>5</v>
+      </c>
+      <c r="P5">
+        <v>5</v>
       </c>
       <c r="Q5" s="6"/>
       <c r="R5" t="b">
@@ -4519,10 +4543,16 @@
         <v>23</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N6">
         <v>2</v>
+      </c>
+      <c r="O6">
+        <v>5</v>
+      </c>
+      <c r="P6">
+        <v>5</v>
       </c>
       <c r="Q6" s="6"/>
       <c r="R6" t="b">
@@ -4564,10 +4594,16 @@
         <v>58</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N7">
         <v>2</v>
+      </c>
+      <c r="O7">
+        <v>5</v>
+      </c>
+      <c r="P7">
+        <v>5</v>
       </c>
       <c r="Q7" s="1"/>
       <c r="R7" t="b">
@@ -4609,10 +4645,16 @@
         <v>58</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N8">
         <v>2</v>
+      </c>
+      <c r="O8">
+        <v>5</v>
+      </c>
+      <c r="P8">
+        <v>5</v>
       </c>
       <c r="Q8" s="6"/>
       <c r="R8" t="b">
@@ -4654,10 +4696,16 @@
         <v>58</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>999</v>
       </c>
       <c r="N9">
         <v>2</v>
+      </c>
+      <c r="O9">
+        <v>5</v>
+      </c>
+      <c r="P9">
+        <v>5</v>
       </c>
       <c r="Q9" s="6"/>
       <c r="R9" t="b">

</xml_diff>